<commit_message>
Document: ui 문서 수정
- ui:0911 ui 정책 문서 보강
- 정책문서: 행동 설계 내용 업데이트
- enenmy: ai를 통한 더미데이터 생성
- spawn: 0908 문서 최신화
</commit_message>
<xml_diff>
--- a/Document/data/enemy.xlsx
+++ b/Document/data/enemy.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git_fork\ProjectShoot\Document\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCF394F-346E-4658-AC8F-FB3557238E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21D3754-6338-4CB5-98C8-BD8DA2A6E4F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="711" firstSheet="1" activeTab="2" xr2:uid="{F9E8F865-F741-4425-897D-555A2E4B3EBE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="711" firstSheet="1" activeTab="1" xr2:uid="{F9E8F865-F741-4425-897D-555A2E4B3EBE}"/>
   </bookViews>
   <sheets>
     <sheet name="깃포크 공부" sheetId="11" state="hidden" r:id="rId1"/>
-    <sheet name="적 일람" sheetId="17" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="20" r:id="rId3"/>
+    <sheet name="적 일람 (기본)" sheetId="22" r:id="rId2"/>
+    <sheet name="적 컨셉" sheetId="23" r:id="rId3"/>
+    <sheet name="적 일람" sheetId="17" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="20" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="271">
   <si>
     <t>no</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -260,13 +262,729 @@
   <si>
     <t>각 영역 안에서 랜덤하게 소환</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enemy_ID</t>
+  </si>
+  <si>
+    <t>Max_HP</t>
+  </si>
+  <si>
+    <t>Move_Speed</t>
+  </si>
+  <si>
+    <t>Collision_Damage</t>
+  </si>
+  <si>
+    <t>Sprite_Name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>E_Yaja_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Yaja_Runner</t>
+  </si>
+  <si>
+    <t>E_Gupsik_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Cafeteria_Ghost</t>
+  </si>
+  <si>
+    <t>E_Maesum_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Bread_Shuttle</t>
+  </si>
+  <si>
+    <t>E_Tardy_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Tardy_Student</t>
+  </si>
+  <si>
+    <t>E_Uniform_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Gym_Clothes</t>
+  </si>
+  <si>
+    <t>E_Backpack_Shield</t>
+  </si>
+  <si>
+    <t>Spr_Heavy_Bag</t>
+  </si>
+  <si>
+    <t>E_Exam_Elite</t>
+  </si>
+  <si>
+    <t>Spr_Exam_Paper</t>
+  </si>
+  <si>
+    <t>E_Monami_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Ballpen_Ghost</t>
+  </si>
+  <si>
+    <t>E_Omr_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Omr_Card</t>
+  </si>
+  <si>
+    <t>E_Fgrade_Elite</t>
+  </si>
+  <si>
+    <t>Spr_F_Bomber</t>
+  </si>
+  <si>
+    <t>E_GroupTask_Shield</t>
+  </si>
+  <si>
+    <t>Spr_Freerider</t>
+  </si>
+  <si>
+    <t>E_Ppt_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Gulim_Ppt</t>
+  </si>
+  <si>
+    <t>E_Usb_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Lost_Usb</t>
+  </si>
+  <si>
+    <t>E_Mt_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Mt_Blackhistory</t>
+  </si>
+  <si>
+    <t>E_Soju_Elite</t>
+  </si>
+  <si>
+    <t>Spr_Fruit_Soju</t>
+  </si>
+  <si>
+    <t>E_Hangover_Shield</t>
+  </si>
+  <si>
+    <t>Spr_Hangover_Drink</t>
+  </si>
+  <si>
+    <t>E_Gwazam_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Smelly_Jacket</t>
+  </si>
+  <si>
+    <t>E_Karaoke_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Coin_Mic</t>
+  </si>
+  <si>
+    <t>E_Pcbang_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Pc_Ramen</t>
+  </si>
+  <si>
+    <t>E_Cupbop_Shield</t>
+  </si>
+  <si>
+    <t>Spr_Noryangjin_Bop</t>
+  </si>
+  <si>
+    <t>E_Goshitel_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Noise_Wall</t>
+  </si>
+  <si>
+    <t>E_Library_Elite</t>
+  </si>
+  <si>
+    <t>Spr_Reserved_Seat</t>
+  </si>
+  <si>
+    <t>E_EnergyDrink_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Caffeine_Monster</t>
+  </si>
+  <si>
+    <t>E_SixAm_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Alarm_Clock</t>
+  </si>
+  <si>
+    <t>E_Subway_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Hell_Subway</t>
+  </si>
+  <si>
+    <t>E_BusDrop_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Stop_Bell</t>
+  </si>
+  <si>
+    <t>E_Earphone_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Tangled_Cord</t>
+  </si>
+  <si>
+    <t>E_PhoneBat_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Battery_1Percent</t>
+  </si>
+  <si>
+    <t>E_Tablet_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Broken_Ipad</t>
+  </si>
+  <si>
+    <t>E_Wifi_Elite</t>
+  </si>
+  <si>
+    <t>Spr_Disconnected_Wi</t>
+  </si>
+  <si>
+    <t>E_Cafe_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Study_Cafe</t>
+  </si>
+  <si>
+    <t>E_Americano_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Spilled_Coffee</t>
+  </si>
+  <si>
+    <t>E_Parttime_Shield</t>
+  </si>
+  <si>
+    <t>Spr_Convenience_GS</t>
+  </si>
+  <si>
+    <t>E_Pos_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Pos_Error</t>
+  </si>
+  <si>
+    <t>E_Delivery_Elite</t>
+  </si>
+  <si>
+    <t>Spr_Bad_Review</t>
+  </si>
+  <si>
+    <t>E_FourCut_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Life_Fourcut</t>
+  </si>
+  <si>
+    <t>E_Tinder_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Dating_App</t>
+  </si>
+  <si>
+    <t>E_Insta_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Story_Viewer</t>
+  </si>
+  <si>
+    <t>E_Reels_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Shorts_Addict</t>
+  </si>
+  <si>
+    <t>E_Diet_Shield</t>
+  </si>
+  <si>
+    <t>Spr_Chicken_Box</t>
+  </si>
+  <si>
+    <t>E_Health_Elite</t>
+  </si>
+  <si>
+    <t>Spr_Dumbbell_Ghost</t>
+  </si>
+  <si>
+    <t>E_Dating_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Cc_Couple</t>
+  </si>
+  <si>
+    <t>E_Breakup_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Midnight_Text</t>
+  </si>
+  <si>
+    <t>E_BlindDate_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Bomb_Drink</t>
+  </si>
+  <si>
+    <t>E_Report_Elite</t>
+  </si>
+  <si>
+    <t>Spr_Plagiarism_Doc</t>
+  </si>
+  <si>
+    <t>E_Tuition_Shield</t>
+  </si>
+  <si>
+    <t>Spr_Tuition_Bill</t>
+  </si>
+  <si>
+    <t>E_Wallet_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Empty_Wallet</t>
+  </si>
+  <si>
+    <t>E_Attend_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Proxy_Student</t>
+  </si>
+  <si>
+    <t>E_Eta_Scout</t>
+  </si>
+  <si>
+    <t>Spr_Community_Troll</t>
+  </si>
+  <si>
+    <t>E_Fossil_Elite</t>
+  </si>
+  <si>
+    <t>Spr_Graduation_Delay</t>
+  </si>
+  <si>
+    <t>id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스프라이트 이름</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Concept</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">야자 시간 도망치는 학생 귀신. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>매우 빠른 속도로 기습하는 1발 컷(20) 자코.</t>
+  </si>
+  <si>
+    <t>무난한 속도의 2발 컷(40) 표준형 잡몹.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">점심시간 급식실로 뛰는 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">매점 빵을 들고 뛰는 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1발(20)에 터지며 쾌적한 타격감을 제공.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">교문이 닫히기 직전 질주하는 지각생. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2발을 버티며 빠르게 하강.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">체육복 빌려가서 안 돌려주는 몽달귀신. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>V자 대형 양날개 배치에 적합.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">전공책으로 가득 찬 무거운 책가방 거북이. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.5초(250)를 버티는 든든한 방패.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">시험지 뭉치가 뭉쳐진 도깨비. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TTK 2초(200)로 유저 화력을 시험하는 중형 몹.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">모나미 볼펜 똥 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1타 컷(20)으로 물량 공세 시 진형을 가득 채우는 용도.</t>
+  </si>
+  <si>
+    <t>OMR 카드 밀려 쓴 원혼.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>느리지만 2발(40)을 버티는 초반 물량전 핵심.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">F학점 폭격기 교수님 그림자. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TTK 2.2초를 요구하며 유저에게 에임 압박.</t>
+  </si>
+  <si>
+    <t>조별과제 무임승차자.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>중형몹 최대 체력(300)으로 3초간 끈질기게 버팀.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">굴림체로 작성된 저주받은 PPT 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1발(20) 컷으로 가볍게 터짐.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">과제 든 USB 잃어버린 원혼. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>최대 속도(250)에 2발 컷으로 심한 기습 압박.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">대학교 MT 장기자랑 흑역사 귀신. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>느린 1발 컷 몹으로 화면 체류 시간 증가.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">달콤한 과일소주 좀비. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TTK 1.8초(180)의 무난한 맷집을 가진 엘리트.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">숙취해소제 골렘. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>체력 280으로 앞선을 막아 플레이어의 동선을 제한함.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">한 달째 안 빤 과잠바 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2발 컷(40)으로 전방위 스폰 시 밸런스 척도.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">코인노래방 마이크 냄새 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1타 컷(20)의 경쾌한 격파 감각 제공.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC방에서 먹다 남은 컵라면 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2발(40)을 버티며 H자 일렬 스폰에 적합.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">노량진 컵밥 떡대 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>최저 속도(80)지만 2.8초를 버티며 탱커 역할을 수행.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">고시원 벽간소음 원혼. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>빠른 속도(230)로 내려오는 1발 컷 유리대포.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">도서관 자리 맡아두고 안 오는 책 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1.8초간 버티는 느릿한 중형 몹.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">밤샘용 고카페인 에너지 드링크 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>속도 최댓값(250)의 돌진형 잡몹.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">아침 6시 알람 소리 악령. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2발 컷(40)에 빠른 속도로 내려와 회피 강제.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2호선 지옥철 좀비 학생. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2타 파괴형(40)으로 대규모 웨이브 시 주력 자코.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">하차벨 안 누르고 화내는 귀신. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1타 파괴(20)의 스탠다드 잡몹.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주머니에서 꼬인 유선 이어폰 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>느린 1발 컷으로 조준 난이도 하락.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>배터리 1% 남은 스마트폰의 불안감.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>빠른 속도(210)로 압박하는 1발 컷 몹.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">액정 박살난 태블릿 귀신. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2발 컷(40)으로 준수한 이동 속도를 가짐.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">수강신청 중 끊긴 와이파이 악령. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>엘리트 몹 중 체력(150)은 낮지만 속도가 빠름.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">카공족(카페 공부) 몽달귀신. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>이동 속도가 낮아 화면에 오래 머무는 2발 컷.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">쏟아진 아이스 아메리카노 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1타 컷(20)의 시원시원한 연출용 자코.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">편의점 알바 괴롭히는 진상 방패. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.5초(250)의 수명을 가진 앞열 고기방패.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">포스기 정산 빵꾸난 원혼. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>적절한 속도의 1발 컷 잡몹.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>설명</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>야식 배달앱 별점 1점 테러범.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1발(20)에 터지며 V자 대형의 꼭짓점 몹으로 좋음.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">네컷사진 엽기 포즈 귀신. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1타 컷(20)이지만 꽤 빠르게 내려옴.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">데이팅 앱 잠수 타는 유령 요괴. </t>
+  </si>
+  <si>
+    <t>2발 컷(40)의 체력을 지닌 표준 몹.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">인스타 스토리 관종 요괴. </t>
+  </si>
+  <si>
+    <t>빠른 기습형 1발 컷(20) 유리대포.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">숏폼 중독으로 뇌가 녹은 귀신. </t>
+  </si>
+  <si>
+    <t>최고 체력(300)과 최저 속도의 완전 탱커.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">야식 치킨의 유혹, 작심삼일 다이어트 트롤. </t>
+  </si>
+  <si>
+    <t>2.4초(240) TTK로 체력이 매우 높은 엘리트.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">닭가슴살만 먹는 헬창 도깨비. </t>
+  </si>
+  <si>
+    <t>1발(20) 파괴 시원한 타격감 담당.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">눈꼴시린 캠퍼스 커플 염장 요괴. </t>
+  </si>
+  <si>
+    <t>2발 컷에 매우 느려 에임 맞추기 쉬움.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">자니...? 이별 후 새벽 감성 원혼. </t>
+  </si>
+  <si>
+    <t>과팅 폭탄주 요괴.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1발(20)에 정확히 파괴되는 엑스트라 잡몹.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2초 TTK(200)의 표준 엘리트 스탯.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">나무위키 긁어온 표절 레포트 요괴. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>최고 체력(300)으로 플레이어 진로 완전 차단.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">등골 빼먹는 등록금 고지서 골렘. </t>
+  </si>
+  <si>
+    <t>1발(20)에 터지지만 빠른 속도로 동체시력 압박.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">월말 텅 빈 텅장 요괴. </t>
+  </si>
+  <si>
+    <t>2발 컷(40)의 안정적인 밸런스를 가진 잡몹.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">대리출석 발각된 귀신. </t>
+  </si>
+  <si>
+    <t>1타(20)에 파괴되는 게임 밸런스의 기본 닻.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">대학 커뮤니티 어그로 관종. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.5초간 데미지를 받아내는 단단한 엘리트.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">졸업을 미룬 암모나이트 화석 선배 좀비. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2초간 화력을 흡수하는(200) 엘리트 기체.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>민준, 서준, 도윤, 예준, 시우, 하준, 지호, 주원, 지훈, 건우, 우진, 선우, 서진, 연우, 유준, 정우, 승우, 은우, 수호, 준우, 태윤, 로운, 윤우, 이안, 지환</t>
+  </si>
+  <si>
+    <t>서연, 서윤, 지우, 서현, 하은, 하윤, 민서, 지유, 윤서, 지민, 채원, 수아, 지아, 다은, 은서, 예은, 소율, 지윤, 하린, 시은, 아윤, 서아, 유나, 가은, 이서</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,6 +1034,15 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -343,12 +1070,51 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -357,7 +1123,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -380,6 +1146,24 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2363,6 +3147,2242 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B604882-023A-4D28-B49D-915BEC004E55}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1:M63"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="20.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5" customWidth="1"/>
+    <col min="10" max="10" width="8.375" customWidth="1"/>
+    <col min="11" max="11" width="21.25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="50.75" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="26.25" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="26.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="4"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+      <c r="F6">
+        <v>220</v>
+      </c>
+      <c r="G6">
+        <v>15</v>
+      </c>
+      <c r="K6" t="s">
+        <v>63</v>
+      </c>
+      <c r="L6" t="s">
+        <v>168</v>
+      </c>
+      <c r="M6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7">
+        <v>40</v>
+      </c>
+      <c r="F7">
+        <v>180</v>
+      </c>
+      <c r="G7">
+        <v>15</v>
+      </c>
+      <c r="K7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L7" t="s">
+        <v>169</v>
+      </c>
+      <c r="M7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
+      </c>
+      <c r="F8">
+        <v>150</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="K8" t="s">
+        <v>67</v>
+      </c>
+      <c r="L8" t="s">
+        <v>172</v>
+      </c>
+      <c r="M8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9">
+        <v>40</v>
+      </c>
+      <c r="F9">
+        <v>200</v>
+      </c>
+      <c r="G9">
+        <v>15</v>
+      </c>
+      <c r="K9" t="s">
+        <v>69</v>
+      </c>
+      <c r="L9" t="s">
+        <v>174</v>
+      </c>
+      <c r="M9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+      <c r="F10">
+        <v>140</v>
+      </c>
+      <c r="G10">
+        <v>10</v>
+      </c>
+      <c r="K10" t="s">
+        <v>71</v>
+      </c>
+      <c r="L10" t="s">
+        <v>176</v>
+      </c>
+      <c r="M10" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11">
+        <v>250</v>
+      </c>
+      <c r="F11">
+        <v>80</v>
+      </c>
+      <c r="G11">
+        <v>30</v>
+      </c>
+      <c r="K11" t="s">
+        <v>73</v>
+      </c>
+      <c r="L11" t="s">
+        <v>178</v>
+      </c>
+      <c r="M11" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12">
+        <v>200</v>
+      </c>
+      <c r="F12">
+        <v>150</v>
+      </c>
+      <c r="G12">
+        <v>25</v>
+      </c>
+      <c r="K12" t="s">
+        <v>75</v>
+      </c>
+      <c r="L12" t="s">
+        <v>180</v>
+      </c>
+      <c r="M12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13">
+        <v>20</v>
+      </c>
+      <c r="F13">
+        <v>160</v>
+      </c>
+      <c r="G13">
+        <v>10</v>
+      </c>
+      <c r="K13" t="s">
+        <v>77</v>
+      </c>
+      <c r="L13" t="s">
+        <v>182</v>
+      </c>
+      <c r="M13" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14">
+        <v>40</v>
+      </c>
+      <c r="F14">
+        <v>130</v>
+      </c>
+      <c r="G14">
+        <v>15</v>
+      </c>
+      <c r="K14" t="s">
+        <v>79</v>
+      </c>
+      <c r="L14" t="s">
+        <v>184</v>
+      </c>
+      <c r="M14" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>10</v>
+      </c>
+      <c r="C15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15">
+        <v>220</v>
+      </c>
+      <c r="F15">
+        <v>120</v>
+      </c>
+      <c r="G15">
+        <v>25</v>
+      </c>
+      <c r="K15" t="s">
+        <v>81</v>
+      </c>
+      <c r="L15" t="s">
+        <v>186</v>
+      </c>
+      <c r="M15" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16">
+        <v>300</v>
+      </c>
+      <c r="F16">
+        <v>85</v>
+      </c>
+      <c r="G16">
+        <v>30</v>
+      </c>
+      <c r="K16" t="s">
+        <v>83</v>
+      </c>
+      <c r="L16" t="s">
+        <v>188</v>
+      </c>
+      <c r="M16" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17">
+        <v>20</v>
+      </c>
+      <c r="F17">
+        <v>150</v>
+      </c>
+      <c r="G17">
+        <v>10</v>
+      </c>
+      <c r="K17" t="s">
+        <v>85</v>
+      </c>
+      <c r="L17" t="s">
+        <v>190</v>
+      </c>
+      <c r="M17" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18">
+        <v>40</v>
+      </c>
+      <c r="F18">
+        <v>250</v>
+      </c>
+      <c r="G18">
+        <v>20</v>
+      </c>
+      <c r="K18" t="s">
+        <v>87</v>
+      </c>
+      <c r="L18" t="s">
+        <v>192</v>
+      </c>
+      <c r="M18" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>14</v>
+      </c>
+      <c r="C19" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19">
+        <v>20</v>
+      </c>
+      <c r="F19">
+        <v>130</v>
+      </c>
+      <c r="G19">
+        <v>10</v>
+      </c>
+      <c r="K19" t="s">
+        <v>89</v>
+      </c>
+      <c r="L19" t="s">
+        <v>194</v>
+      </c>
+      <c r="M19" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>15</v>
+      </c>
+      <c r="C20" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20">
+        <v>180</v>
+      </c>
+      <c r="F20">
+        <v>140</v>
+      </c>
+      <c r="G20">
+        <v>20</v>
+      </c>
+      <c r="K20" t="s">
+        <v>91</v>
+      </c>
+      <c r="L20" t="s">
+        <v>196</v>
+      </c>
+      <c r="M20" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>92</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21">
+        <v>280</v>
+      </c>
+      <c r="F21">
+        <v>90</v>
+      </c>
+      <c r="G21">
+        <v>30</v>
+      </c>
+      <c r="K21" t="s">
+        <v>93</v>
+      </c>
+      <c r="L21" t="s">
+        <v>198</v>
+      </c>
+      <c r="M21" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>94</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E22">
+        <v>40</v>
+      </c>
+      <c r="F22">
+        <v>170</v>
+      </c>
+      <c r="G22">
+        <v>15</v>
+      </c>
+      <c r="K22" t="s">
+        <v>95</v>
+      </c>
+      <c r="L22" t="s">
+        <v>200</v>
+      </c>
+      <c r="M22" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E23">
+        <v>20</v>
+      </c>
+      <c r="F23">
+        <v>180</v>
+      </c>
+      <c r="G23">
+        <v>10</v>
+      </c>
+      <c r="K23" t="s">
+        <v>97</v>
+      </c>
+      <c r="L23" t="s">
+        <v>202</v>
+      </c>
+      <c r="M23" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>19</v>
+      </c>
+      <c r="C24" t="s">
+        <v>98</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24">
+        <v>40</v>
+      </c>
+      <c r="F24">
+        <v>120</v>
+      </c>
+      <c r="G24">
+        <v>15</v>
+      </c>
+      <c r="K24" t="s">
+        <v>99</v>
+      </c>
+      <c r="L24" t="s">
+        <v>204</v>
+      </c>
+      <c r="M24" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s">
+        <v>100</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25">
+        <v>280</v>
+      </c>
+      <c r="F25">
+        <v>80</v>
+      </c>
+      <c r="G25">
+        <v>30</v>
+      </c>
+      <c r="K25" t="s">
+        <v>101</v>
+      </c>
+      <c r="L25" t="s">
+        <v>206</v>
+      </c>
+      <c r="M25" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>21</v>
+      </c>
+      <c r="C26" t="s">
+        <v>102</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E26">
+        <v>20</v>
+      </c>
+      <c r="F26">
+        <v>230</v>
+      </c>
+      <c r="G26">
+        <v>15</v>
+      </c>
+      <c r="K26" t="s">
+        <v>103</v>
+      </c>
+      <c r="L26" t="s">
+        <v>208</v>
+      </c>
+      <c r="M26" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>22</v>
+      </c>
+      <c r="C27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E27">
+        <v>180</v>
+      </c>
+      <c r="F27">
+        <v>110</v>
+      </c>
+      <c r="G27">
+        <v>20</v>
+      </c>
+      <c r="K27" t="s">
+        <v>105</v>
+      </c>
+      <c r="L27" t="s">
+        <v>210</v>
+      </c>
+      <c r="M27" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>23</v>
+      </c>
+      <c r="C28" t="s">
+        <v>106</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E28">
+        <v>20</v>
+      </c>
+      <c r="F28">
+        <v>250</v>
+      </c>
+      <c r="G28">
+        <v>15</v>
+      </c>
+      <c r="K28" t="s">
+        <v>107</v>
+      </c>
+      <c r="L28" t="s">
+        <v>212</v>
+      </c>
+      <c r="M28" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>24</v>
+      </c>
+      <c r="C29" t="s">
+        <v>108</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E29">
+        <v>40</v>
+      </c>
+      <c r="F29">
+        <v>200</v>
+      </c>
+      <c r="G29">
+        <v>20</v>
+      </c>
+      <c r="K29" t="s">
+        <v>109</v>
+      </c>
+      <c r="L29" t="s">
+        <v>214</v>
+      </c>
+      <c r="M29" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>25</v>
+      </c>
+      <c r="C30" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30">
+        <v>40</v>
+      </c>
+      <c r="F30">
+        <v>140</v>
+      </c>
+      <c r="G30">
+        <v>15</v>
+      </c>
+      <c r="K30" t="s">
+        <v>111</v>
+      </c>
+      <c r="L30" t="s">
+        <v>216</v>
+      </c>
+      <c r="M30" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>26</v>
+      </c>
+      <c r="C31" t="s">
+        <v>112</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E31">
+        <v>20</v>
+      </c>
+      <c r="F31">
+        <v>160</v>
+      </c>
+      <c r="G31">
+        <v>10</v>
+      </c>
+      <c r="K31" t="s">
+        <v>113</v>
+      </c>
+      <c r="L31" t="s">
+        <v>218</v>
+      </c>
+      <c r="M31" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
+        <v>27</v>
+      </c>
+      <c r="C32" t="s">
+        <v>114</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E32">
+        <v>20</v>
+      </c>
+      <c r="F32">
+        <v>130</v>
+      </c>
+      <c r="G32">
+        <v>10</v>
+      </c>
+      <c r="K32" t="s">
+        <v>115</v>
+      </c>
+      <c r="L32" t="s">
+        <v>220</v>
+      </c>
+      <c r="M32" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>28</v>
+      </c>
+      <c r="C33" t="s">
+        <v>116</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E33">
+        <v>20</v>
+      </c>
+      <c r="F33">
+        <v>210</v>
+      </c>
+      <c r="G33">
+        <v>15</v>
+      </c>
+      <c r="K33" t="s">
+        <v>117</v>
+      </c>
+      <c r="L33" t="s">
+        <v>222</v>
+      </c>
+      <c r="M33" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>29</v>
+      </c>
+      <c r="C34" t="s">
+        <v>118</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34">
+        <v>40</v>
+      </c>
+      <c r="F34">
+        <v>150</v>
+      </c>
+      <c r="G34">
+        <v>15</v>
+      </c>
+      <c r="K34" t="s">
+        <v>119</v>
+      </c>
+      <c r="L34" t="s">
+        <v>224</v>
+      </c>
+      <c r="M34" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
+        <v>30</v>
+      </c>
+      <c r="C35" t="s">
+        <v>120</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E35">
+        <v>150</v>
+      </c>
+      <c r="F35">
+        <v>180</v>
+      </c>
+      <c r="G35">
+        <v>20</v>
+      </c>
+      <c r="K35" t="s">
+        <v>121</v>
+      </c>
+      <c r="L35" t="s">
+        <v>226</v>
+      </c>
+      <c r="M35" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
+        <v>31</v>
+      </c>
+      <c r="C36" t="s">
+        <v>122</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E36">
+        <v>40</v>
+      </c>
+      <c r="F36">
+        <v>120</v>
+      </c>
+      <c r="G36">
+        <v>15</v>
+      </c>
+      <c r="K36" t="s">
+        <v>123</v>
+      </c>
+      <c r="L36" t="s">
+        <v>228</v>
+      </c>
+      <c r="M36" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>32</v>
+      </c>
+      <c r="C37" t="s">
+        <v>124</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E37">
+        <v>20</v>
+      </c>
+      <c r="F37">
+        <v>150</v>
+      </c>
+      <c r="G37">
+        <v>10</v>
+      </c>
+      <c r="K37" t="s">
+        <v>125</v>
+      </c>
+      <c r="L37" t="s">
+        <v>230</v>
+      </c>
+      <c r="M37" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
+        <v>33</v>
+      </c>
+      <c r="C38" t="s">
+        <v>126</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E38">
+        <v>250</v>
+      </c>
+      <c r="F38">
+        <v>90</v>
+      </c>
+      <c r="G38">
+        <v>30</v>
+      </c>
+      <c r="K38" t="s">
+        <v>127</v>
+      </c>
+      <c r="L38" t="s">
+        <v>232</v>
+      </c>
+      <c r="M38" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>34</v>
+      </c>
+      <c r="C39" t="s">
+        <v>128</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E39">
+        <v>20</v>
+      </c>
+      <c r="F39">
+        <v>170</v>
+      </c>
+      <c r="G39">
+        <v>10</v>
+      </c>
+      <c r="K39" t="s">
+        <v>129</v>
+      </c>
+      <c r="L39" t="s">
+        <v>234</v>
+      </c>
+      <c r="M39" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>35</v>
+      </c>
+      <c r="C40" t="s">
+        <v>130</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E40">
+        <v>200</v>
+      </c>
+      <c r="F40">
+        <v>130</v>
+      </c>
+      <c r="G40">
+        <v>25</v>
+      </c>
+      <c r="K40" t="s">
+        <v>131</v>
+      </c>
+      <c r="L40" t="s">
+        <v>268</v>
+      </c>
+      <c r="M40" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>36</v>
+      </c>
+      <c r="C41" t="s">
+        <v>132</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E41">
+        <v>20</v>
+      </c>
+      <c r="F41">
+        <v>150</v>
+      </c>
+      <c r="G41">
+        <v>10</v>
+      </c>
+      <c r="K41" t="s">
+        <v>133</v>
+      </c>
+      <c r="L41" t="s">
+        <v>237</v>
+      </c>
+      <c r="M41" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>37</v>
+      </c>
+      <c r="C42" t="s">
+        <v>134</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E42">
+        <v>20</v>
+      </c>
+      <c r="F42">
+        <v>190</v>
+      </c>
+      <c r="G42">
+        <v>10</v>
+      </c>
+      <c r="K42" t="s">
+        <v>135</v>
+      </c>
+      <c r="L42" t="s">
+        <v>239</v>
+      </c>
+      <c r="M42" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>38</v>
+      </c>
+      <c r="C43" t="s">
+        <v>136</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E43">
+        <v>40</v>
+      </c>
+      <c r="F43">
+        <v>150</v>
+      </c>
+      <c r="G43">
+        <v>15</v>
+      </c>
+      <c r="K43" t="s">
+        <v>137</v>
+      </c>
+      <c r="L43" t="s">
+        <v>241</v>
+      </c>
+      <c r="M43" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A44" s="1">
+        <v>39</v>
+      </c>
+      <c r="C44" t="s">
+        <v>138</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E44">
+        <v>20</v>
+      </c>
+      <c r="F44">
+        <v>220</v>
+      </c>
+      <c r="G44">
+        <v>15</v>
+      </c>
+      <c r="K44" t="s">
+        <v>139</v>
+      </c>
+      <c r="L44" t="s">
+        <v>243</v>
+      </c>
+      <c r="M44" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A45" s="1">
+        <v>40</v>
+      </c>
+      <c r="C45" t="s">
+        <v>140</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E45">
+        <v>300</v>
+      </c>
+      <c r="F45">
+        <v>80</v>
+      </c>
+      <c r="G45">
+        <v>30</v>
+      </c>
+      <c r="K45" t="s">
+        <v>141</v>
+      </c>
+      <c r="L45" t="s">
+        <v>245</v>
+      </c>
+      <c r="M45" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
+        <v>41</v>
+      </c>
+      <c r="C46" t="s">
+        <v>142</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E46">
+        <v>240</v>
+      </c>
+      <c r="F46">
+        <v>120</v>
+      </c>
+      <c r="G46">
+        <v>25</v>
+      </c>
+      <c r="K46" t="s">
+        <v>143</v>
+      </c>
+      <c r="L46" t="s">
+        <v>247</v>
+      </c>
+      <c r="M46" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A47" s="1">
+        <v>42</v>
+      </c>
+      <c r="C47" t="s">
+        <v>144</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E47">
+        <v>20</v>
+      </c>
+      <c r="F47">
+        <v>150</v>
+      </c>
+      <c r="G47">
+        <v>10</v>
+      </c>
+      <c r="K47" t="s">
+        <v>145</v>
+      </c>
+      <c r="L47" t="s">
+        <v>249</v>
+      </c>
+      <c r="M47" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A48" s="1">
+        <v>43</v>
+      </c>
+      <c r="C48" t="s">
+        <v>146</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E48">
+        <v>40</v>
+      </c>
+      <c r="F48">
+        <v>110</v>
+      </c>
+      <c r="G48">
+        <v>15</v>
+      </c>
+      <c r="K48" t="s">
+        <v>147</v>
+      </c>
+      <c r="L48" t="s">
+        <v>251</v>
+      </c>
+      <c r="M48" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
+        <v>44</v>
+      </c>
+      <c r="C49" t="s">
+        <v>148</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E49">
+        <v>20</v>
+      </c>
+      <c r="F49">
+        <v>160</v>
+      </c>
+      <c r="G49">
+        <v>10</v>
+      </c>
+      <c r="K49" t="s">
+        <v>149</v>
+      </c>
+      <c r="L49" t="s">
+        <v>254</v>
+      </c>
+      <c r="M49" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>45</v>
+      </c>
+      <c r="C50" t="s">
+        <v>150</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E50">
+        <v>200</v>
+      </c>
+      <c r="F50">
+        <v>150</v>
+      </c>
+      <c r="G50">
+        <v>25</v>
+      </c>
+      <c r="K50" t="s">
+        <v>151</v>
+      </c>
+      <c r="L50" t="s">
+        <v>255</v>
+      </c>
+      <c r="M50" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
+        <v>46</v>
+      </c>
+      <c r="C51" t="s">
+        <v>152</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E51">
+        <v>300</v>
+      </c>
+      <c r="F51">
+        <v>95</v>
+      </c>
+      <c r="G51">
+        <v>30</v>
+      </c>
+      <c r="K51" t="s">
+        <v>153</v>
+      </c>
+      <c r="L51" t="s">
+        <v>257</v>
+      </c>
+      <c r="M51" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
+        <v>47</v>
+      </c>
+      <c r="C52" t="s">
+        <v>154</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E52">
+        <v>20</v>
+      </c>
+      <c r="F52">
+        <v>200</v>
+      </c>
+      <c r="G52">
+        <v>15</v>
+      </c>
+      <c r="K52" t="s">
+        <v>155</v>
+      </c>
+      <c r="L52" t="s">
+        <v>259</v>
+      </c>
+      <c r="M52" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A53" s="1">
+        <v>48</v>
+      </c>
+      <c r="C53" t="s">
+        <v>156</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E53">
+        <v>40</v>
+      </c>
+      <c r="F53">
+        <v>140</v>
+      </c>
+      <c r="G53">
+        <v>15</v>
+      </c>
+      <c r="K53" t="s">
+        <v>157</v>
+      </c>
+      <c r="L53" t="s">
+        <v>261</v>
+      </c>
+      <c r="M53" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
+        <v>49</v>
+      </c>
+      <c r="C54" t="s">
+        <v>158</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E54">
+        <v>20</v>
+      </c>
+      <c r="F54">
+        <v>150</v>
+      </c>
+      <c r="G54">
+        <v>10</v>
+      </c>
+      <c r="K54" t="s">
+        <v>159</v>
+      </c>
+      <c r="L54" t="s">
+        <v>263</v>
+      </c>
+      <c r="M54" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A55" s="1">
+        <v>50</v>
+      </c>
+      <c r="C55" t="s">
+        <v>160</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E55">
+        <v>250</v>
+      </c>
+      <c r="F55">
+        <v>100</v>
+      </c>
+      <c r="G55">
+        <v>25</v>
+      </c>
+      <c r="K55" t="s">
+        <v>161</v>
+      </c>
+      <c r="L55" t="s">
+        <v>265</v>
+      </c>
+      <c r="M55" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="L58" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B63" s="13"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C77AADE4-AB87-44A7-9D24-4E88A390DA88}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1:G63"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="41.25" customWidth="1"/>
+    <col min="4" max="4" width="50.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="26.25" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="26.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="G5" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D6" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7" t="s">
+        <v>169</v>
+      </c>
+      <c r="G7" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>171</v>
+      </c>
+      <c r="D8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>173</v>
+      </c>
+      <c r="D9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>175</v>
+      </c>
+      <c r="D10" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>177</v>
+      </c>
+      <c r="D11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D12" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D13" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>183</v>
+      </c>
+      <c r="D14" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>10</v>
+      </c>
+      <c r="C15" t="s">
+        <v>185</v>
+      </c>
+      <c r="D15" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D16" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>189</v>
+      </c>
+      <c r="D17" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>191</v>
+      </c>
+      <c r="D18" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>14</v>
+      </c>
+      <c r="C19" t="s">
+        <v>193</v>
+      </c>
+      <c r="D19" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>15</v>
+      </c>
+      <c r="C20" t="s">
+        <v>195</v>
+      </c>
+      <c r="D20" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>197</v>
+      </c>
+      <c r="D21" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>199</v>
+      </c>
+      <c r="D22" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>18</v>
+      </c>
+      <c r="C23" t="s">
+        <v>201</v>
+      </c>
+      <c r="D23" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>19</v>
+      </c>
+      <c r="C24" t="s">
+        <v>203</v>
+      </c>
+      <c r="D24" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s">
+        <v>205</v>
+      </c>
+      <c r="D25" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>21</v>
+      </c>
+      <c r="C26" t="s">
+        <v>207</v>
+      </c>
+      <c r="D26" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>22</v>
+      </c>
+      <c r="C27" t="s">
+        <v>209</v>
+      </c>
+      <c r="D27" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>23</v>
+      </c>
+      <c r="C28" t="s">
+        <v>211</v>
+      </c>
+      <c r="D28" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>24</v>
+      </c>
+      <c r="C29" t="s">
+        <v>213</v>
+      </c>
+      <c r="D29" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>25</v>
+      </c>
+      <c r="C30" t="s">
+        <v>215</v>
+      </c>
+      <c r="D30" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>26</v>
+      </c>
+      <c r="C31" t="s">
+        <v>217</v>
+      </c>
+      <c r="D31" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
+        <v>27</v>
+      </c>
+      <c r="C32" t="s">
+        <v>219</v>
+      </c>
+      <c r="D32" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>28</v>
+      </c>
+      <c r="C33" t="s">
+        <v>221</v>
+      </c>
+      <c r="D33" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>29</v>
+      </c>
+      <c r="C34" t="s">
+        <v>223</v>
+      </c>
+      <c r="D34" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
+        <v>30</v>
+      </c>
+      <c r="C35" t="s">
+        <v>225</v>
+      </c>
+      <c r="D35" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
+        <v>31</v>
+      </c>
+      <c r="C36" t="s">
+        <v>227</v>
+      </c>
+      <c r="D36" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>32</v>
+      </c>
+      <c r="C37" t="s">
+        <v>229</v>
+      </c>
+      <c r="D37" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
+        <v>33</v>
+      </c>
+      <c r="C38" t="s">
+        <v>231</v>
+      </c>
+      <c r="D38" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>34</v>
+      </c>
+      <c r="C39" t="s">
+        <v>233</v>
+      </c>
+      <c r="D39" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>35</v>
+      </c>
+      <c r="C40" t="s">
+        <v>236</v>
+      </c>
+      <c r="D40" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>36</v>
+      </c>
+      <c r="C41" t="s">
+        <v>238</v>
+      </c>
+      <c r="D41" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>37</v>
+      </c>
+      <c r="C42" t="s">
+        <v>240</v>
+      </c>
+      <c r="D42" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>38</v>
+      </c>
+      <c r="C43" t="s">
+        <v>242</v>
+      </c>
+      <c r="D43" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="1">
+        <v>39</v>
+      </c>
+      <c r="C44" t="s">
+        <v>244</v>
+      </c>
+      <c r="D44" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="1">
+        <v>40</v>
+      </c>
+      <c r="C45" t="s">
+        <v>246</v>
+      </c>
+      <c r="D45" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
+        <v>41</v>
+      </c>
+      <c r="C46" t="s">
+        <v>248</v>
+      </c>
+      <c r="D46" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="1">
+        <v>42</v>
+      </c>
+      <c r="C47" t="s">
+        <v>250</v>
+      </c>
+      <c r="D47" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="1">
+        <v>43</v>
+      </c>
+      <c r="C48" t="s">
+        <v>252</v>
+      </c>
+      <c r="D48" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
+        <v>44</v>
+      </c>
+      <c r="C49" t="s">
+        <v>253</v>
+      </c>
+      <c r="D49" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>45</v>
+      </c>
+      <c r="C50" t="s">
+        <v>256</v>
+      </c>
+      <c r="D50" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
+        <v>46</v>
+      </c>
+      <c r="C51" t="s">
+        <v>258</v>
+      </c>
+      <c r="D51" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
+        <v>47</v>
+      </c>
+      <c r="C52" t="s">
+        <v>260</v>
+      </c>
+      <c r="D52" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="1">
+        <v>48</v>
+      </c>
+      <c r="C53" t="s">
+        <v>262</v>
+      </c>
+      <c r="D53" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
+        <v>49</v>
+      </c>
+      <c r="C54" t="s">
+        <v>264</v>
+      </c>
+      <c r="D54" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="1">
+        <v>50</v>
+      </c>
+      <c r="C55" t="s">
+        <v>266</v>
+      </c>
+      <c r="D55" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D58" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B63" s="13"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96250C9B-AC9A-4D12-8447-AA0DC8C1E6CA}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
@@ -2552,7 +5572,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9726223E-47D7-4B21-B2EE-18763D410474}">
   <dimension ref="B2:H35"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>

</xml_diff>